<commit_message>
feat/FSEL-6178: sửa format của excel báo cáo tiến độ học tập
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ManagerReports/BaoCaoTienDoV1.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ManagerReports/BaoCaoTienDoV1.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ManagerReports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haqua\source\repos\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ManagerReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{287F7ED9-8703-4FF4-A84E-AB739DF409C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3966D29-FAFF-4A31-A697-B04684A3ADD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F30A999D-8AA9-4EB0-A60C-86C78673A0AD}"/>
+    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15720" xr2:uid="{F30A999D-8AA9-4EB0-A60C-86C78673A0AD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="179021" concurrentCalc="0"/>
+  <calcPr calcId="179021"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -106,11 +106,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -156,8 +156,26 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -194,7 +212,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -276,11 +294,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -298,20 +355,25 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -639,32 +701,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C8AE389-ADB7-4203-A796-E150C4B1ABD0}">
   <dimension ref="A1:CM6"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="7" width="17.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.25" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="23.125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="24.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="37.25" customWidth="1"/>
+    <col min="1" max="6" width="9.140625" style="14"/>
+    <col min="7" max="7" width="17.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.28515625" style="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="37.28515625" style="14" customWidth="1"/>
+    <col min="14" max="91" width="9.140625" style="14"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:91" ht="26.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
       <c r="M1" s="1" t="s">
         <v>16</v>
       </c>
@@ -748,14 +812,14 @@
       <c r="CM1" s="2"/>
     </row>
     <row r="2" spans="1:91" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
       <c r="G2" s="4" t="s">
         <v>19</v>
       </c>
@@ -853,14 +917,14 @@
       <c r="CM2" s="2"/>
     </row>
     <row r="3" spans="1:91" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
       <c r="G3" s="6">
         <v>0</v>
       </c>
@@ -1050,217 +1114,217 @@
       <c r="CL4" s="2"/>
       <c r="CM4" s="2"/>
     </row>
-    <row r="5" spans="1:91" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+    <row r="5" spans="1:91" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="I5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="11" t="s">
+      <c r="J5" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="K5" s="10" t="s">
+      <c r="K5" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="10" t="s">
+      <c r="L5" s="11" t="s">
         <v>9</v>
       </c>
       <c r="M5" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
-      <c r="P5" s="13"/>
-      <c r="Q5" s="13"/>
-      <c r="R5" s="13"/>
-      <c r="S5" s="13"/>
-      <c r="T5" s="13"/>
-      <c r="U5" s="13"/>
-      <c r="V5" s="13"/>
-      <c r="W5" s="13"/>
-      <c r="X5" s="13"/>
-      <c r="Y5" s="13"/>
-      <c r="Z5" s="13"/>
-      <c r="AA5" s="13"/>
-      <c r="AB5" s="13"/>
-      <c r="AC5" s="13"/>
-      <c r="AD5" s="13"/>
-      <c r="AE5" s="13"/>
-      <c r="AF5" s="13"/>
-      <c r="AG5" s="13"/>
-      <c r="AH5" s="13"/>
-      <c r="AI5" s="13"/>
-      <c r="AJ5" s="13"/>
-      <c r="AK5" s="13"/>
-      <c r="AL5" s="13"/>
-      <c r="AM5" s="13"/>
-      <c r="AN5" s="13"/>
-      <c r="AO5" s="13"/>
-      <c r="AP5" s="13"/>
-      <c r="AQ5" s="13"/>
-      <c r="AR5" s="13"/>
-      <c r="AS5" s="13"/>
-      <c r="AT5" s="13"/>
-      <c r="AU5" s="13"/>
-      <c r="AV5" s="13"/>
-      <c r="AW5" s="13"/>
-      <c r="AX5" s="13"/>
-      <c r="AY5" s="13"/>
-      <c r="AZ5" s="13"/>
-      <c r="BA5" s="13"/>
-      <c r="BB5" s="13"/>
-      <c r="BC5" s="13"/>
-      <c r="BD5" s="13"/>
-      <c r="BE5" s="13"/>
-      <c r="BF5" s="13"/>
-      <c r="BG5" s="13"/>
-      <c r="BH5" s="13"/>
-      <c r="BI5" s="13"/>
-      <c r="BJ5" s="13"/>
-      <c r="BK5" s="13"/>
-      <c r="BL5" s="13"/>
-      <c r="BM5" s="13"/>
-      <c r="BN5" s="13"/>
-      <c r="BO5" s="13"/>
-      <c r="BP5" s="13"/>
-      <c r="BQ5" s="13"/>
-      <c r="BR5" s="13"/>
-      <c r="BS5" s="13"/>
-      <c r="BT5" s="13"/>
-      <c r="BU5" s="13"/>
-      <c r="BV5" s="13"/>
-      <c r="BW5" s="13"/>
-      <c r="BX5" s="13"/>
-      <c r="BY5" s="13"/>
-      <c r="BZ5" s="13"/>
-      <c r="CA5" s="13"/>
-      <c r="CB5" s="13"/>
-      <c r="CC5" s="13"/>
-      <c r="CD5" s="13"/>
-      <c r="CE5" s="13"/>
-      <c r="CF5" s="13"/>
-      <c r="CG5" s="13"/>
-      <c r="CH5" s="13"/>
-      <c r="CI5" s="13"/>
-      <c r="CJ5" s="13"/>
-      <c r="CK5" s="13"/>
-      <c r="CL5" s="13"/>
-      <c r="CM5" s="13"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+      <c r="P5" s="9"/>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="9"/>
+      <c r="S5" s="9"/>
+      <c r="T5" s="9"/>
+      <c r="U5" s="9"/>
+      <c r="V5" s="9"/>
+      <c r="W5" s="9"/>
+      <c r="X5" s="9"/>
+      <c r="Y5" s="9"/>
+      <c r="Z5" s="9"/>
+      <c r="AA5" s="9"/>
+      <c r="AB5" s="9"/>
+      <c r="AC5" s="9"/>
+      <c r="AD5" s="9"/>
+      <c r="AE5" s="9"/>
+      <c r="AF5" s="9"/>
+      <c r="AG5" s="9"/>
+      <c r="AH5" s="9"/>
+      <c r="AI5" s="9"/>
+      <c r="AJ5" s="9"/>
+      <c r="AK5" s="9"/>
+      <c r="AL5" s="9"/>
+      <c r="AM5" s="9"/>
+      <c r="AN5" s="9"/>
+      <c r="AO5" s="9"/>
+      <c r="AP5" s="9"/>
+      <c r="AQ5" s="9"/>
+      <c r="AR5" s="9"/>
+      <c r="AS5" s="9"/>
+      <c r="AT5" s="9"/>
+      <c r="AU5" s="9"/>
+      <c r="AV5" s="9"/>
+      <c r="AW5" s="9"/>
+      <c r="AX5" s="9"/>
+      <c r="AY5" s="9"/>
+      <c r="AZ5" s="9"/>
+      <c r="BA5" s="9"/>
+      <c r="BB5" s="9"/>
+      <c r="BC5" s="9"/>
+      <c r="BD5" s="9"/>
+      <c r="BE5" s="9"/>
+      <c r="BF5" s="9"/>
+      <c r="BG5" s="9"/>
+      <c r="BH5" s="9"/>
+      <c r="BI5" s="9"/>
+      <c r="BJ5" s="9"/>
+      <c r="BK5" s="9"/>
+      <c r="BL5" s="9"/>
+      <c r="BM5" s="9"/>
+      <c r="BN5" s="9"/>
+      <c r="BO5" s="9"/>
+      <c r="BP5" s="9"/>
+      <c r="BQ5" s="9"/>
+      <c r="BR5" s="9"/>
+      <c r="BS5" s="9"/>
+      <c r="BT5" s="9"/>
+      <c r="BU5" s="9"/>
+      <c r="BV5" s="9"/>
+      <c r="BW5" s="9"/>
+      <c r="BX5" s="9"/>
+      <c r="BY5" s="9"/>
+      <c r="BZ5" s="9"/>
+      <c r="CA5" s="9"/>
+      <c r="CB5" s="9"/>
+      <c r="CC5" s="9"/>
+      <c r="CD5" s="9"/>
+      <c r="CE5" s="9"/>
+      <c r="CF5" s="9"/>
+      <c r="CG5" s="9"/>
+      <c r="CH5" s="9"/>
+      <c r="CI5" s="9"/>
+      <c r="CJ5" s="9"/>
+      <c r="CK5" s="9"/>
+      <c r="CL5" s="9"/>
+      <c r="CM5" s="9"/>
     </row>
-    <row r="6" spans="1:91" ht="15" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="2"/>
-      <c r="T6" s="2"/>
-      <c r="U6" s="2"/>
-      <c r="V6" s="2"/>
-      <c r="W6" s="2"/>
-      <c r="X6" s="2"/>
-      <c r="Y6" s="2"/>
-      <c r="Z6" s="2"/>
-      <c r="AA6" s="2"/>
-      <c r="AB6" s="2"/>
-      <c r="AC6" s="2"/>
-      <c r="AD6" s="2"/>
-      <c r="AE6" s="2"/>
-      <c r="AF6" s="2"/>
-      <c r="AG6" s="2"/>
-      <c r="AH6" s="2"/>
-      <c r="AI6" s="2"/>
-      <c r="AJ6" s="2"/>
-      <c r="AK6" s="2"/>
-      <c r="AL6" s="2"/>
-      <c r="AM6" s="2"/>
-      <c r="AN6" s="2"/>
-      <c r="AO6" s="2"/>
-      <c r="AP6" s="2"/>
-      <c r="AQ6" s="2"/>
-      <c r="AR6" s="2"/>
-      <c r="AS6" s="2"/>
-      <c r="AT6" s="2"/>
-      <c r="AU6" s="2"/>
-      <c r="AV6" s="2"/>
-      <c r="AW6" s="2"/>
-      <c r="AX6" s="2"/>
-      <c r="AY6" s="2"/>
-      <c r="AZ6" s="2"/>
-      <c r="BA6" s="2"/>
-      <c r="BB6" s="2"/>
-      <c r="BC6" s="2"/>
-      <c r="BD6" s="2"/>
-      <c r="BE6" s="2"/>
-      <c r="BF6" s="2"/>
-      <c r="BG6" s="2"/>
-      <c r="BH6" s="2"/>
-      <c r="BI6" s="2"/>
-      <c r="BJ6" s="2"/>
-      <c r="BK6" s="2"/>
-      <c r="BL6" s="2"/>
-      <c r="BM6" s="2"/>
-      <c r="BN6" s="2"/>
-      <c r="BO6" s="2"/>
-      <c r="BP6" s="2"/>
-      <c r="BQ6" s="2"/>
-      <c r="BR6" s="2"/>
-      <c r="BS6" s="2"/>
-      <c r="BT6" s="2"/>
-      <c r="BU6" s="2"/>
-      <c r="BV6" s="2"/>
-      <c r="BW6" s="2"/>
-      <c r="BX6" s="2"/>
-      <c r="BY6" s="2"/>
-      <c r="BZ6" s="2"/>
-      <c r="CA6" s="2"/>
-      <c r="CB6" s="2"/>
-      <c r="CC6" s="2"/>
-      <c r="CD6" s="2"/>
-      <c r="CE6" s="2"/>
-      <c r="CF6" s="2"/>
-      <c r="CG6" s="2"/>
-      <c r="CH6" s="2"/>
-      <c r="CI6" s="2"/>
-      <c r="CJ6" s="2"/>
-      <c r="CK6" s="2"/>
-      <c r="CL6" s="2"/>
-      <c r="CM6" s="2"/>
+    <row r="6" spans="1:91" x14ac:dyDescent="0.25">
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="13"/>
+      <c r="M6" s="13"/>
+      <c r="N6" s="13"/>
+      <c r="O6" s="13"/>
+      <c r="P6" s="13"/>
+      <c r="Q6" s="13"/>
+      <c r="R6" s="13"/>
+      <c r="S6" s="13"/>
+      <c r="T6" s="13"/>
+      <c r="U6" s="13"/>
+      <c r="V6" s="13"/>
+      <c r="W6" s="13"/>
+      <c r="X6" s="13"/>
+      <c r="Y6" s="13"/>
+      <c r="Z6" s="13"/>
+      <c r="AA6" s="13"/>
+      <c r="AB6" s="13"/>
+      <c r="AC6" s="13"/>
+      <c r="AD6" s="13"/>
+      <c r="AE6" s="13"/>
+      <c r="AF6" s="13"/>
+      <c r="AG6" s="13"/>
+      <c r="AH6" s="13"/>
+      <c r="AI6" s="13"/>
+      <c r="AJ6" s="13"/>
+      <c r="AK6" s="13"/>
+      <c r="AL6" s="13"/>
+      <c r="AM6" s="13"/>
+      <c r="AN6" s="13"/>
+      <c r="AO6" s="13"/>
+      <c r="AP6" s="13"/>
+      <c r="AQ6" s="13"/>
+      <c r="AR6" s="13"/>
+      <c r="AS6" s="13"/>
+      <c r="AT6" s="13"/>
+      <c r="AU6" s="13"/>
+      <c r="AV6" s="13"/>
+      <c r="AW6" s="13"/>
+      <c r="AX6" s="13"/>
+      <c r="AY6" s="13"/>
+      <c r="AZ6" s="13"/>
+      <c r="BA6" s="13"/>
+      <c r="BB6" s="13"/>
+      <c r="BC6" s="13"/>
+      <c r="BD6" s="13"/>
+      <c r="BE6" s="13"/>
+      <c r="BF6" s="13"/>
+      <c r="BG6" s="13"/>
+      <c r="BH6" s="13"/>
+      <c r="BI6" s="13"/>
+      <c r="BJ6" s="13"/>
+      <c r="BK6" s="13"/>
+      <c r="BL6" s="13"/>
+      <c r="BM6" s="13"/>
+      <c r="BN6" s="13"/>
+      <c r="BO6" s="13"/>
+      <c r="BP6" s="13"/>
+      <c r="BQ6" s="13"/>
+      <c r="BR6" s="13"/>
+      <c r="BS6" s="13"/>
+      <c r="BT6" s="13"/>
+      <c r="BU6" s="13"/>
+      <c r="BV6" s="13"/>
+      <c r="BW6" s="13"/>
+      <c r="BX6" s="13"/>
+      <c r="BY6" s="13"/>
+      <c r="BZ6" s="13"/>
+      <c r="CA6" s="13"/>
+      <c r="CB6" s="13"/>
+      <c r="CC6" s="13"/>
+      <c r="CD6" s="13"/>
+      <c r="CE6" s="13"/>
+      <c r="CF6" s="13"/>
+      <c r="CG6" s="13"/>
+      <c r="CH6" s="13"/>
+      <c r="CI6" s="13"/>
+      <c r="CJ6" s="13"/>
+      <c r="CK6" s="13"/>
+      <c r="CL6" s="13"/>
+      <c r="CM6" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1274,11 +1338,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="9c5e610e-28db-44df-ba41-c446aaffe434" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1509,27 +1574,17 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="9c5e610e-28db-44df-ba41-c446aaffe434" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2805DAB0-0287-4ED8-AE35-4ED06A772265}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{018B28C1-B173-45F8-AB6D-10704E690C54}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="9c5e610e-28db-44df-ba41-c446aaffe434"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="e78f2374-cb69-45b5-92b0-6a1f828922e7"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1554,9 +1609,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{018B28C1-B173-45F8-AB6D-10704E690C54}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2805DAB0-0287-4ED8-AE35-4ED06A772265}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="9c5e610e-28db-44df-ba41-c446aaffe434"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="e78f2374-cb69-45b5-92b0-6a1f828922e7"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>